<commit_message>
updating excel and plotting code
</commit_message>
<xml_diff>
--- a/src/fungi_pipeline/excel/fungal_summary.xlsx
+++ b/src/fungi_pipeline/excel/fungal_summary.xlsx
@@ -33,7 +33,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,11 @@
         <fgColor rgb="00FF6347"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0087CEFA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -63,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -77,6 +82,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -445,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z14"/>
+  <dimension ref="A1:AD14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -474,11 +482,13 @@
     <col width="16" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr"/>
-      <c r="B1" t="inlineStr"/>
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>AMR</t>
@@ -511,82 +521,97 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Biofilm</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Biofilm</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Biofilm</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Biofilm</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Biofilm</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Biofilm</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Biofilm</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Biofilm</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Biofilm</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Hpat</t>
+          <t>H-pat</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Hpat</t>
+          <t>H-pat</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>H-pat</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>H-pat</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>Thermophile</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>Rad-res</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>Spore</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Spore</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Spore</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Spore</t>
         </is>
       </c>
     </row>
@@ -603,213 +628,497 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>ERG11-Candida-albicans</t>
+          <t>ERG11</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>CDR1-Candida-albicans</t>
+          <t>CDR1</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>MDR1-Candida-albicans</t>
+          <t>MDR1</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>UPC2-Candida-albicans</t>
+          <t>UPC2</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>TAC1-Candida-albicans</t>
+          <t>TAC1</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>MRR1-Candida-albicans</t>
+          <t>MRR1</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t>BCR1-Candida-albicans</t>
+          <t>BCR1</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>EFG1-Candida-albicans</t>
+          <t>EFG1</t>
         </is>
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>TEC1-Candida-albicans</t>
+          <t>TEC1</t>
         </is>
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>HWP1-Candida-albicans</t>
+          <t>HWP1</t>
         </is>
       </c>
       <c r="M2" s="1" t="inlineStr">
         <is>
-          <t>ALS3-Candida-albicans</t>
+          <t>ALS3</t>
         </is>
       </c>
       <c r="N2" s="1" t="inlineStr">
         <is>
-          <t>NDT80-Candida-albicans</t>
+          <t>NDT80</t>
         </is>
       </c>
       <c r="O2" s="1" t="inlineStr">
         <is>
-          <t>ERG251-Candida-albicans</t>
+          <t>ERG251</t>
         </is>
       </c>
       <c r="P2" s="1" t="inlineStr">
         <is>
-          <t>CZF1-Candida-albicans</t>
+          <t>CZF1</t>
         </is>
       </c>
       <c r="Q2" s="1" t="inlineStr">
         <is>
-          <t>FLO8-Candida-albicans</t>
+          <t>FLO8</t>
         </is>
       </c>
       <c r="R2" s="1" t="inlineStr">
         <is>
-          <t>SAP5-Candida-albicans</t>
+          <t>SAP5</t>
         </is>
       </c>
       <c r="S2" s="1" t="inlineStr">
         <is>
-          <t>RIM101-Candida-albicans</t>
+          <t>PLB1</t>
         </is>
       </c>
       <c r="T2" s="1" t="inlineStr">
         <is>
-          <t>HSP90-Aspergillus-fumigatus</t>
+          <t>LAC1</t>
         </is>
       </c>
       <c r="U2" s="1" t="inlineStr">
         <is>
-          <t>brlA-Emericella-nidulans</t>
+          <t>RIM101</t>
         </is>
       </c>
       <c r="V2" s="1" t="inlineStr">
         <is>
-          <t>abaA-Emericella-nidulans</t>
+          <t>HSP90</t>
         </is>
       </c>
       <c r="W2" s="1" t="inlineStr">
         <is>
-          <t>wetA-Emericella-nidulans</t>
+          <t>RAD51</t>
         </is>
       </c>
       <c r="X2" s="1" t="inlineStr">
         <is>
-          <t>srr1-Coprinopsis-cinerea</t>
-        </is>
-      </c>
-      <c r="Y2" s="2" t="inlineStr">
+          <t>brlA</t>
+        </is>
+      </c>
+      <c r="Y2" s="1" t="inlineStr">
+        <is>
+          <t>abaA</t>
+        </is>
+      </c>
+      <c r="Z2" s="1" t="inlineStr">
+        <is>
+          <t>wetA</t>
+        </is>
+      </c>
+      <c r="AA2" s="1" t="inlineStr">
+        <is>
+          <t>srr1</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>r,y,r+y</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr">
-        <is>
-          <t>Phylum</t>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>Phyla</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="S3" s="1" t="inlineStr">
+        <is>
+          <t>Cryptococcus</t>
+        </is>
+      </c>
+      <c r="T3" s="1" t="inlineStr">
+        <is>
+          <t>Cryptococcus</t>
+        </is>
+      </c>
+      <c r="U3" s="1" t="inlineStr">
+        <is>
+          <t>Candida</t>
+        </is>
+      </c>
+      <c r="V3" s="1" t="inlineStr">
+        <is>
+          <t>Aspergillus</t>
+        </is>
+      </c>
+      <c r="W3" s="1" t="inlineStr">
+        <is>
+          <t>Saccharomyces</t>
+        </is>
+      </c>
+      <c r="X3" s="1" t="inlineStr">
+        <is>
+          <t>Emericella</t>
+        </is>
+      </c>
+      <c r="Y3" s="1" t="inlineStr">
+        <is>
+          <t>Emericella</t>
+        </is>
+      </c>
+      <c r="Z3" s="1" t="inlineStr">
+        <is>
+          <t>Emericella</t>
+        </is>
+      </c>
+      <c r="AA3" s="1" t="inlineStr">
+        <is>
+          <t>Coprinopsis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="M4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="O4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="P4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="Q4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="R4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="S4" s="1" t="inlineStr">
+        <is>
+          <t>Neoformans</t>
+        </is>
+      </c>
+      <c r="T4" s="1" t="inlineStr">
+        <is>
+          <t>Neoformans</t>
+        </is>
+      </c>
+      <c r="U4" s="1" t="inlineStr">
+        <is>
+          <t>Albicans</t>
+        </is>
+      </c>
+      <c r="V4" s="1" t="inlineStr">
+        <is>
+          <t>Fumigatus</t>
+        </is>
+      </c>
+      <c r="W4" s="1" t="inlineStr">
+        <is>
+          <t>Cerevisiae</t>
+        </is>
+      </c>
+      <c r="X4" s="1" t="inlineStr">
+        <is>
+          <t>Nidulans</t>
+        </is>
+      </c>
+      <c r="Y4" s="1" t="inlineStr">
+        <is>
+          <t>Nidulans</t>
+        </is>
+      </c>
+      <c r="Z4" s="1" t="inlineStr">
+        <is>
+          <t>Nidulans</t>
+        </is>
+      </c>
+      <c r="AA4" s="1" t="inlineStr">
+        <is>
+          <t>Cinerea</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Yamadazyma tenuis</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B5" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C5" s="5" t="n">
         <v>71.8</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D5" s="5" t="n">
         <v>69.8</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>55.9</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F5" s="5" t="n">
         <v>58.7</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G5" s="5" t="n">
         <v>49</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H5" s="5" t="n">
         <v>51.2</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>85.5</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="J5" s="5" t="n">
         <v>51.7</v>
       </c>
-      <c r="K3" s="5" t="n">
+      <c r="K5" s="5" t="n">
         <v>58.1</v>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="L5" s="5" t="n">
         <v>52.7</v>
       </c>
-      <c r="M3" s="5" t="n">
+      <c r="M5" s="5" t="n">
         <v>41.5</v>
       </c>
-      <c r="N3" s="5" t="n">
+      <c r="N5" s="5" t="n">
         <v>63.8</v>
       </c>
-      <c r="O3" s="5" t="n">
+      <c r="O5" s="5" t="n">
         <v>66.8</v>
       </c>
-      <c r="P3" s="5" t="n">
+      <c r="P5" s="5" t="n">
         <v>59.6</v>
       </c>
-      <c r="Q3" s="5" t="n">
+      <c r="Q5" s="5" t="n">
         <v>38.7</v>
       </c>
-      <c r="R3" s="5" t="n">
+      <c r="R5" s="5" t="n">
         <v>37.6</v>
       </c>
-      <c r="S3" s="5" t="n">
+      <c r="S5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="5" t="n">
         <v>68.8</v>
       </c>
-      <c r="T3" s="5" t="n">
+      <c r="V5" s="5" t="n">
         <v>74.5</v>
       </c>
-      <c r="U3" s="5" t="n">
+      <c r="W5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="V3" s="5" t="n">
+      <c r="Y5" s="5" t="n">
         <v>47.7</v>
       </c>
-      <c r="W3" s="5" t="n">
+      <c r="Z5" s="5" t="n">
         <v>40.6</v>
       </c>
-      <c r="X3" s="5" t="n">
+      <c r="AA5" s="5" t="n">
         <v>44.4</v>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>1,21,22</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr">
         <is>
           <t>Ascomycota</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Summary Statistics</t>
         </is>

</xml_diff>